<commit_message>
feat(excel): a unit column, and no capitulo total across units
Task 2.5, the workbook half. The budget sheet gains a Unit column after
Metrado: each partida states the unit its total is in, as the category
criterion resolved it ("Partida carries its unit"), and each line and
capitulo does too. A capitulo is totalled only when its partidas share
one unit; one that grouping split by unit states no total rather than
one adding m2 to u ("Incompatible units are not summed").

The three reference workbooks were regenerated with the tool the suite
keeps for it (METRADO_REGENERATE_GOLDENS=1); the only change in them is
the Unit column, read back cell by cell before committing.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Metrado.Excel.Tests/Goldens/empty-result.xlsx
+++ b/tests/Metrado.Excel.Tests/Goldens/empty-result.xlsx
@@ -33,6 +33,9 @@
   </x:si>
   <x:si>
     <x:t>Metrado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Unit</x:t>
   </x:si>
   <x:si>
     <x:t>Boundary mode</x:t>
@@ -401,10 +404,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F2"/>
+  <x:dimension ref="A1:G2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="1" spans="1:6">
+    <x:row r="1" spans="1:7">
       <x:c r="A1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -412,7 +415,7 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:6">
+    <x:row r="2" spans="1:7">
       <x:c r="A2" s="0" t="s">
         <x:v>1</x:v>
       </x:c>
@@ -430,6 +433,9 @@
       </x:c>
       <x:c r="F2" s="0" t="s">
         <x:v>6</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>7</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -451,12 +457,12 @@
   <x:sheetData>
     <x:row r="1" spans="1:4">
       <x:c r="A1" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
       <x:c r="A2" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B2" s="0">
         <x:v>0</x:v>
@@ -467,13 +473,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>